<commit_message>
fixid some git problems
</commit_message>
<xml_diff>
--- a/docs/weekly-mini-projects/weekly-mini-project-02/evaluation/Weekly_Mini_Project_02_Team_2_Leader_Evaluation.xlsx
+++ b/docs/weekly-mini-projects/weekly-mini-project-02/evaluation/Weekly_Mini_Project_02_Team_2_Leader_Evaluation.xlsx
@@ -1,39 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nawarhisso/Documents/Training/BootCamp/repositories/b4f-cohort8-salamiyah-react-node-bootcamp-2026/docs/Weekly Mini Projects/weekly-mini-project-01/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\B4f\BootCamp\b4f-cohort8-salamiyah-next-nest-bootcamp-2026\docs\weekly-mini-projects\weekly-mini-project-02\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF4EA4A-BC04-C040-82B4-16BBE1F509BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D6A6ED-A34B-4629-92C1-69AE829F7020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evaluation" sheetId="1" r:id="rId1"/>
     <sheet name="Criteria Guide" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="83">
   <si>
     <t>Weekly Mini Project 02 — Leader Evaluation of Team Members</t>
   </si>
@@ -228,6 +216,60 @@
   </si>
   <si>
     <t>Excellent</t>
+  </si>
+  <si>
+    <t>Backend development</t>
+  </si>
+  <si>
+    <t>He did as expected of him, tried to keep me informed of every step he takes, tried to be available as much as he can.</t>
+  </si>
+  <si>
+    <t>Teamwork instead of individual work, he is used to do everything alone. Be more flexible. He is initiative a lot, he could try fix something even if it's not his job</t>
+  </si>
+  <si>
+    <t>He is a good partner, could be annoying at some point, but he alwayes make things right at the end.</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>He did what he could do in the time which he had, easy to get advices from him.</t>
+  </si>
+  <si>
+    <t>presentation skills just.</t>
+  </si>
+  <si>
+    <t>one of the best</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>He did as expected of him and more, helped his teammates when they needed.</t>
+  </si>
+  <si>
+    <t>To be less initiative.</t>
+  </si>
+  <si>
+    <t>God of Astra</t>
+  </si>
+  <si>
+    <t>She did what she was told to do without delay, keeped me informed with everything she did, a good contributer.</t>
+  </si>
+  <si>
+    <t>Nothing in mind.</t>
+  </si>
+  <si>
+    <t>A lovelly addition to any team</t>
+  </si>
+  <si>
+    <t>He tried his best, and tried to keep involved in the work.</t>
+  </si>
+  <si>
+    <t>To be more initiative.</t>
+  </si>
+  <si>
+    <t>Nothing</t>
   </si>
 </sst>
 </file>
@@ -238,7 +280,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -488,7 +530,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -792,9 +834,9 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" customWidth="1"/>
+    <col min="1" max="1" width="8.125" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="17" width="13" customWidth="1"/>
     <col min="18" max="18" width="11" customWidth="1"/>
@@ -853,7 +895,7 @@
       <c r="U2" s="23"/>
       <c r="V2" s="23"/>
     </row>
-    <row r="3" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
@@ -972,7 +1014,7 @@
       <c r="U10" s="25"/>
       <c r="V10" s="26"/>
     </row>
-    <row r="11" spans="1:22" ht="62" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" ht="62.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
@@ -1047,29 +1089,67 @@
       <c r="B12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="9" t="str">
+      <c r="C12" s="8">
+        <v>5</v>
+      </c>
+      <c r="D12" s="8">
+        <v>4</v>
+      </c>
+      <c r="E12" s="8">
+        <v>4</v>
+      </c>
+      <c r="F12" s="8">
+        <v>5</v>
+      </c>
+      <c r="G12" s="8">
+        <v>4</v>
+      </c>
+      <c r="H12" s="8">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8">
+        <v>4</v>
+      </c>
+      <c r="J12" s="8">
+        <v>2</v>
+      </c>
+      <c r="K12" s="8">
+        <v>3</v>
+      </c>
+      <c r="L12" s="8">
+        <v>5</v>
+      </c>
+      <c r="M12" s="8">
+        <v>3</v>
+      </c>
+      <c r="N12" s="8">
+        <v>5</v>
+      </c>
+      <c r="O12" s="8">
+        <v>4</v>
+      </c>
+      <c r="P12" s="8">
+        <v>4</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>4</v>
+      </c>
+      <c r="R12" s="9">
         <f>IF(COUNT(C12:Q12)=0,"",AVERAGE(C12:Q12))</f>
-        <v/>
-      </c>
-      <c r="S12" s="10"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="10"/>
-      <c r="V12" s="10"/>
+        <v>4.0666666666666664</v>
+      </c>
+      <c r="S12" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="T12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="U12" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="V12" s="10" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="13" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
@@ -1078,29 +1158,67 @@
       <c r="B13" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="9" t="str">
+      <c r="C13" s="11">
+        <v>4</v>
+      </c>
+      <c r="D13" s="11">
+        <v>4</v>
+      </c>
+      <c r="E13" s="11">
+        <v>4</v>
+      </c>
+      <c r="F13" s="11">
+        <v>5</v>
+      </c>
+      <c r="G13" s="11">
+        <v>5</v>
+      </c>
+      <c r="H13" s="11">
+        <v>4</v>
+      </c>
+      <c r="I13" s="11">
+        <v>5</v>
+      </c>
+      <c r="J13" s="11">
+        <v>4</v>
+      </c>
+      <c r="K13" s="11">
+        <v>4</v>
+      </c>
+      <c r="L13" s="11">
+        <v>5</v>
+      </c>
+      <c r="M13" s="11">
+        <v>5</v>
+      </c>
+      <c r="N13" s="11">
+        <v>4</v>
+      </c>
+      <c r="O13" s="11">
+        <v>5</v>
+      </c>
+      <c r="P13" s="11">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="11">
+        <v>4</v>
+      </c>
+      <c r="R13" s="9">
         <f>IF(COUNT(C13:Q13)=0,"",AVERAGE(C13:Q13))</f>
-        <v/>
-      </c>
-      <c r="S13" s="12"/>
-      <c r="T13" s="12"/>
-      <c r="U13" s="12"/>
-      <c r="V13" s="12"/>
+        <v>4.333333333333333</v>
+      </c>
+      <c r="S13" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="T13" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="U13" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="V13" s="12" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="14" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
@@ -1109,29 +1227,67 @@
       <c r="B14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
-      <c r="M14" s="8"/>
-      <c r="N14" s="8"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="9" t="str">
+      <c r="C14" s="8">
+        <v>5</v>
+      </c>
+      <c r="D14" s="8">
+        <v>5</v>
+      </c>
+      <c r="E14" s="8">
+        <v>4</v>
+      </c>
+      <c r="F14" s="8">
+        <v>5</v>
+      </c>
+      <c r="G14" s="8">
+        <v>4</v>
+      </c>
+      <c r="H14" s="8">
+        <v>5</v>
+      </c>
+      <c r="I14" s="8">
+        <v>4</v>
+      </c>
+      <c r="J14" s="8">
+        <v>5</v>
+      </c>
+      <c r="K14" s="8">
+        <v>5</v>
+      </c>
+      <c r="L14" s="8">
+        <v>5</v>
+      </c>
+      <c r="M14" s="8">
+        <v>5</v>
+      </c>
+      <c r="N14" s="8">
+        <v>5</v>
+      </c>
+      <c r="O14" s="8">
+        <v>4</v>
+      </c>
+      <c r="P14" s="8">
+        <v>5</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>5</v>
+      </c>
+      <c r="R14" s="9">
         <f>IF(COUNT(C14:Q14)=0,"",AVERAGE(C14:Q14))</f>
-        <v/>
-      </c>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="10"/>
-      <c r="V14" s="10"/>
+        <v>4.7333333333333334</v>
+      </c>
+      <c r="S14" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="T14" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="U14" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="V14" s="10" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="15" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
@@ -1140,29 +1296,67 @@
       <c r="B15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="9" t="str">
+      <c r="C15" s="11">
+        <v>4</v>
+      </c>
+      <c r="D15" s="11">
+        <v>5</v>
+      </c>
+      <c r="E15" s="11">
+        <v>5</v>
+      </c>
+      <c r="F15" s="11">
+        <v>5</v>
+      </c>
+      <c r="G15" s="11">
+        <v>4</v>
+      </c>
+      <c r="H15" s="11">
+        <v>5</v>
+      </c>
+      <c r="I15" s="11">
+        <v>4</v>
+      </c>
+      <c r="J15" s="11">
+        <v>5</v>
+      </c>
+      <c r="K15" s="11">
+        <v>4</v>
+      </c>
+      <c r="L15" s="11">
+        <v>5</v>
+      </c>
+      <c r="M15" s="11">
+        <v>5</v>
+      </c>
+      <c r="N15" s="11">
+        <v>5</v>
+      </c>
+      <c r="O15" s="11">
+        <v>3</v>
+      </c>
+      <c r="P15" s="11">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="11">
+        <v>5</v>
+      </c>
+      <c r="R15" s="9">
         <f>IF(COUNT(C15:Q15)=0,"",AVERAGE(C15:Q15))</f>
-        <v/>
-      </c>
-      <c r="S15" s="12"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="12"/>
-      <c r="V15" s="12"/>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="S15" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="T15" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="U15" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="V15" s="12" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="16" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
@@ -1171,29 +1365,67 @@
       <c r="B16" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="9" t="str">
+      <c r="C16" s="8">
+        <v>4</v>
+      </c>
+      <c r="D16" s="8">
+        <v>4</v>
+      </c>
+      <c r="E16" s="8">
+        <v>3</v>
+      </c>
+      <c r="F16" s="8">
+        <v>3</v>
+      </c>
+      <c r="G16" s="8">
+        <v>4</v>
+      </c>
+      <c r="H16" s="8">
+        <v>3</v>
+      </c>
+      <c r="I16" s="8">
+        <v>3</v>
+      </c>
+      <c r="J16" s="8">
+        <v>5</v>
+      </c>
+      <c r="K16" s="8">
+        <v>4</v>
+      </c>
+      <c r="L16" s="8">
+        <v>3</v>
+      </c>
+      <c r="M16" s="8">
+        <v>5</v>
+      </c>
+      <c r="N16" s="8">
+        <v>5</v>
+      </c>
+      <c r="O16" s="8">
+        <v>4</v>
+      </c>
+      <c r="P16" s="8">
+        <v>4</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>4</v>
+      </c>
+      <c r="R16" s="9">
         <f>IF(COUNT(C16:Q16)=0,"",AVERAGE(C16:Q16))</f>
-        <v/>
-      </c>
-      <c r="S16" s="10"/>
-      <c r="T16" s="10"/>
-      <c r="U16" s="10"/>
-      <c r="V16" s="10"/>
+        <v>3.8666666666666667</v>
+      </c>
+      <c r="S16" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="T16" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="U16" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="V16" s="10" t="s">
+        <v>82</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1224,7 +1456,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -1245,7 +1477,7 @@
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
     </row>
-    <row r="3" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
@@ -1307,7 +1539,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="28" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A10" s="13">
         <v>5</v>
       </c>
@@ -1373,7 +1605,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="28" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A16" s="13">
         <v>11</v>
       </c>
@@ -1428,7 +1660,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="B22" s="19" t="s">
         <v>59</v>
       </c>

</xml_diff>